<commit_message>
Change old functions in new style
</commit_message>
<xml_diff>
--- a/work_with_prepared_data/datas/control/02.02.2023_n_12.xlsx
+++ b/work_with_prepared_data/datas/control/02.02.2023_n_12.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Scripts\neuro_stats\work_with_prepared_data\datas\control\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\neuro_stats\work_with_prepared_data\datas\control\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{489C1EEF-C602-4EAA-A55E-09CD962A3965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="26520" windowHeight="9165"/>
+    <workbookView xWindow="7470" yWindow="3585" windowWidth="17895" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -125,9 +126,6 @@
     <t>2,3 - 1,8 - 1,0</t>
   </si>
   <si>
-    <t>1,8 - 1,4 - 1,8</t>
-  </si>
-  <si>
     <t>2,2 - 1,7 - 1,1</t>
   </si>
   <si>
@@ -252,12 +250,15 @@
   </si>
   <si>
     <t>2,8 - 2,0 - 1,6</t>
+  </si>
+  <si>
+    <t>1,8 - 1,4 - 0,8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -569,7 +570,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -636,28 +637,28 @@
         <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -671,28 +672,28 @@
         <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -706,28 +707,28 @@
         <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -741,13 +742,13 @@
         <v>31</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G6" t="s">
         <v>19</v>
@@ -759,10 +760,10 @@
         <v>19</v>
       </c>
       <c r="J6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -779,7 +780,7 @@
         <v>30</v>
       </c>
       <c r="E7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F7">
         <v>0.3</v>
@@ -811,28 +812,28 @@
         <v>32</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -843,31 +844,31 @@
         <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>75</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G9" t="s">
         <v>29</v>
       </c>
       <c r="H9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>